<commit_message>
tạo RIR cho phép cập nhật code do QC kiểm tra
</commit_message>
<xml_diff>
--- a/MPR_Managerment/Templates/pnk_template.xlsx
+++ b/MPR_Managerment/Templates/pnk_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c02630c4a1efac79/Working/Final_Project_DLHI_Management/MPR_Managerment/Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{05A4B9D2-E5DF-4680-9B59-691B1ADD956A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A852ADF9-978E-4CB9-A168-665E43D5EC25}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="8_{05A4B9D2-E5DF-4680-9B59-691B1ADD956A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{174C5697-8E3E-473A-9A49-AE39E40AA669}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{3CBA7E04-0AAE-4902-83D7-5F527B47C979}"/>
   </bookViews>
@@ -754,6 +754,24 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="5" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="2" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -772,6 +790,9 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="15" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -800,27 +821,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="5" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="18" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="2" borderId="17" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="11" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="3" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="3" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1884,18 +1884,18 @@
       <c r="F5" s="6"/>
     </row>
     <row r="6" spans="1:254" ht="69" customHeight="1">
-      <c r="A6" s="80" t="s">
+      <c r="A6" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="81"/>
-      <c r="C6" s="81"/>
-      <c r="D6" s="81"/>
-      <c r="E6" s="81"/>
-      <c r="F6" s="81"/>
-      <c r="G6" s="81"/>
-      <c r="H6" s="81"/>
-      <c r="I6" s="81"/>
-      <c r="J6" s="81"/>
+      <c r="B6" s="87"/>
+      <c r="C6" s="87"/>
+      <c r="D6" s="87"/>
+      <c r="E6" s="87"/>
+      <c r="F6" s="87"/>
+      <c r="G6" s="87"/>
+      <c r="H6" s="87"/>
+      <c r="I6" s="87"/>
+      <c r="J6" s="87"/>
     </row>
     <row r="7" spans="1:254" s="14" customFormat="1" ht="34.5" customHeight="1" thickBot="1">
       <c r="A7" s="9"/>
@@ -1919,20 +1919,20 @@
       <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="95" t="s">
+      <c r="C8" s="88" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="95"/>
+      <c r="D8" s="88"/>
       <c r="E8" s="16"/>
-      <c r="F8" s="82" t="s">
+      <c r="F8" s="89" t="s">
         <v>9</v>
       </c>
-      <c r="G8" s="83"/>
-      <c r="H8" s="86" t="s">
+      <c r="G8" s="90"/>
+      <c r="H8" s="93" t="s">
         <v>10</v>
       </c>
-      <c r="I8" s="87"/>
-      <c r="J8" s="90" t="s">
+      <c r="I8" s="94"/>
+      <c r="J8" s="97" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1946,11 +1946,11 @@
       </c>
       <c r="D9" s="17"/>
       <c r="E9" s="7"/>
-      <c r="F9" s="84"/>
-      <c r="G9" s="85"/>
-      <c r="H9" s="88"/>
-      <c r="I9" s="89"/>
-      <c r="J9" s="91"/>
+      <c r="F9" s="91"/>
+      <c r="G9" s="92"/>
+      <c r="H9" s="95"/>
+      <c r="I9" s="96"/>
+      <c r="J9" s="98"/>
       <c r="K9" s="18"/>
       <c r="L9" s="18"/>
       <c r="M9" s="18"/>
@@ -2198,13 +2198,13 @@
     </row>
     <row r="10" spans="1:254" s="2" customFormat="1" ht="23.25" customHeight="1">
       <c r="A10" s="17"/>
-      <c r="B10" s="96" t="s">
+      <c r="B10" s="76" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="97" t="s">
+      <c r="C10" s="77" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="98"/>
+      <c r="D10" s="78"/>
       <c r="E10" s="7"/>
       <c r="F10" s="19"/>
       <c r="G10" s="20"/>
@@ -3261,10 +3261,10 @@
     <row r="15" spans="1:254" s="34" customFormat="1" ht="19.2" customHeight="1">
       <c r="A15" s="29"/>
       <c r="B15" s="30"/>
-      <c r="C15" s="76" t="s">
+      <c r="C15" s="82" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="77"/>
+      <c r="D15" s="83"/>
       <c r="E15" s="31" t="s">
         <v>28</v>
       </c>
@@ -3287,13 +3287,13 @@
       <c r="J16" s="40"/>
     </row>
     <row r="17" spans="1:249" s="44" customFormat="1" ht="36.75" customHeight="1">
-      <c r="A17" s="78" t="s">
+      <c r="A17" s="84" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="79"/>
-      <c r="C17" s="79"/>
-      <c r="D17" s="79"/>
-      <c r="E17" s="79"/>
+      <c r="B17" s="85"/>
+      <c r="C17" s="85"/>
+      <c r="D17" s="85"/>
+      <c r="E17" s="85"/>
       <c r="F17" s="41"/>
       <c r="G17" s="42"/>
       <c r="H17" s="43"/>
@@ -4324,8 +4324,8 @@
       <c r="C21" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="D21" s="92"/>
-      <c r="E21" s="92"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="79"/>
       <c r="F21" s="59"/>
       <c r="G21" s="56"/>
       <c r="H21" s="51"/>
@@ -4583,8 +4583,8 @@
       </c>
       <c r="D22" s="62"/>
       <c r="E22" s="63"/>
-      <c r="F22" s="93"/>
-      <c r="G22" s="94"/>
+      <c r="F22" s="80"/>
+      <c r="G22" s="81"/>
       <c r="H22" s="51"/>
       <c r="I22" s="51"/>
       <c r="J22" s="51"/>
@@ -4838,8 +4838,8 @@
       <c r="C23" s="63"/>
       <c r="D23" s="62"/>
       <c r="E23" s="63"/>
-      <c r="F23" s="93"/>
-      <c r="G23" s="94"/>
+      <c r="F23" s="80"/>
+      <c r="G23" s="81"/>
       <c r="H23" s="51"/>
       <c r="I23" s="51"/>
       <c r="J23" s="51"/>
@@ -5888,19 +5888,19 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="F8:G9"/>
+    <mergeCell ref="H8:I9"/>
+    <mergeCell ref="J8:J9"/>
     <mergeCell ref="D21:E21"/>
     <mergeCell ref="F22:G22"/>
     <mergeCell ref="F23:G23"/>
     <mergeCell ref="C15:D15"/>
     <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="C8:D8"/>
-    <mergeCell ref="F8:G9"/>
-    <mergeCell ref="H8:I9"/>
-    <mergeCell ref="J8:J9"/>
   </mergeCells>
   <pageMargins left="0.49" right="0.25" top="0.32" bottom="0.28999999999999998" header="0.42" footer="0.3"/>
-  <pageSetup paperSize="9" scale="51" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="53" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>